<commit_message>
Import/Export forecast and stavilised v1
</commit_message>
<xml_diff>
--- a/app/templates/report/forecast.xlsx
+++ b/app/templates/report/forecast.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774B8F21-A814-4461-8184-958C6ADAD086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0615B13-CD71-4E90-8933-1252030F5E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -118,11 +118,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="#,##0\ &quot;€&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="mm/yyyy"/>
-    <numFmt numFmtId="167" formatCode="#,##0%;[Red]\-#,##0%"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="#,##0%;[Red]\-#,##0%"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -171,7 +170,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -196,8 +195,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -249,9 +254,20 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color theme="0" tint="-0.34998626667073579"/>
       </left>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -262,28 +278,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="15" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -292,10 +311,14 @@
   </cellStyles>
   <dxfs count="1">
     <dxf>
+      <font>
+        <strike val="0"/>
+      </font>
       <border>
-        <top style="thin">
+        <top style="hair">
           <color auto="1"/>
         </top>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
@@ -686,110 +709,110 @@
   <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" style="3" customWidth="1"/>
     <col min="2" max="2" width="14.140625" style="1" customWidth="1"/>
     <col min="3" max="11" width="11.85546875" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="14.42578125" style="1"/>
+    <col min="12" max="12" width="10.28515625" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="14.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="L1" s="2" t="e">
+      <c r="L1" s="13" t="e">
         <f>YEAR(A3)</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="12">
+      <c r="B3" s="10"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="15">
         <f>1-SUM(D3:F3)</f>
         <v>1</v>
       </c>
-      <c r="H3" s="11"/>
       <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="12"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="A3:K3">
+  <conditionalFormatting sqref="A3:K99999">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$B3&lt;&gt;$B1</formula>
+      <formula>$A2&gt;$A3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Import/Export forecast and stabilised v2
</commit_message>
<xml_diff>
--- a/app/templates/report/forecast.xlsx
+++ b/app/templates/report/forecast.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0615B13-CD71-4E90-8933-1252030F5E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60154366-B3F6-4D8A-8BA7-DB27B5190A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Resource</t>
   </si>
@@ -93,9 +93,6 @@
   </si>
   <si>
     <t>Rent_short</t>
-  </si>
-  <si>
-    <t>Rent_group</t>
   </si>
   <si>
     <t>Services</t>
@@ -724,7 +721,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>1</v>
@@ -748,7 +745,7 @@
         <v>8</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L1" s="13" t="e">
         <f>YEAR(A3)</f>
@@ -774,17 +771,15 @@
       <c r="F2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Import/Export forecast and stabilised fix 1
</commit_message>
<xml_diff>
--- a/app/templates/report/forecast.xlsx
+++ b/app/templates/report/forecast.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60154366-B3F6-4D8A-8BA7-DB27B5190A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B68A918-7AF6-4001-ADF7-404F3790A929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -167,18 +167,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="22"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -278,15 +272,12 @@
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="15" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="15" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -299,7 +290,10 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -706,101 +700,101 @@
   <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.140625" style="1" customWidth="1"/>
     <col min="3" max="11" width="11.85546875" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.28515625" style="1" customWidth="1"/>
     <col min="13" max="16384" width="14.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:12" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="13" t="e">
+      <c r="L1" s="12" t="e">
         <f>YEAR(A3)</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="15">
+      <c r="B3" s="9"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="14">
         <f>1-SUM(D3:F3)</f>
         <v>1</v>
       </c>
-      <c r="I3" s="11"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="12"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Import/Export forecast and stabilised v3
</commit_message>
<xml_diff>
--- a/app/templates/report/forecast.xlsx
+++ b/app/templates/report/forecast.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30790696-942A-4AB8-BF74-8C5FAA44E566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261C2CD3-CC80-4863-9B3E-CFE98C8F03C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Resource</t>
   </si>
@@ -116,6 +116,12 @@
   </si>
   <si>
     <t>Discount</t>
+  </si>
+  <si>
+    <t>Forecast beds</t>
+  </si>
+  <si>
+    <t>Beds</t>
   </si>
 </sst>
 </file>
@@ -276,7 +282,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -301,6 +307,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -704,17 +711,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" style="1" customWidth="1"/>
-    <col min="3" max="12" width="11.85546875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="10.28515625" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="14.42578125" style="1"/>
+    <col min="2" max="3" width="14.140625" style="1" customWidth="1"/>
+    <col min="4" max="13" width="11.85546875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="14.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -722,41 +729,44 @@
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="12" t="e">
+      <c r="N1" s="12" t="e">
         <f>YEAR(A3)</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
@@ -764,56 +774,60 @@
         <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="4"/>
+      <c r="I2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="9"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="8"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="7"/>
       <c r="F3" s="8"/>
-      <c r="G3" s="14">
-        <f>1-SUM(D3:F3)</f>
+      <c r="G3" s="8"/>
+      <c r="H3" s="14">
+        <f>1-SUM(E3:G3)</f>
         <v>1</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="11"/>
+      <c r="I3" s="8"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="A3:L99999">
+  <conditionalFormatting sqref="A3:M99999">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$A2&gt;$A3</formula>
     </cfRule>
@@ -821,7 +835,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <ignoredErrors>
-    <ignoredError sqref="M1" evalError="1"/>
+    <ignoredError sqref="N1" evalError="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Import/Export forecast and stabilised v4
</commit_message>
<xml_diff>
--- a/app/templates/report/forecast.xlsx
+++ b/app/templates/report/forecast.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261C2CD3-CC80-4863-9B3E-CFE98C8F03C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51DEE2AD-6704-4BCE-8251-1D6B539DB7E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Forecast" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Forecast!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Forecast!$A$1:$AA$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
   <si>
     <t>Resource</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Final cleaning</t>
   </si>
   <si>
-    <t>Reinvoices</t>
-  </si>
-  <si>
     <t>Date_price</t>
   </si>
   <si>
@@ -105,10 +102,6 @@
   </si>
   <si>
     <t>% Occup.</t>
-  </si>
-  <si>
-    <t>Total
-Reinvoices</t>
   </si>
   <si>
     <t>%
@@ -122,18 +115,85 @@
   </si>
   <si>
     <t>Beds</t>
+  </si>
+  <si>
+    <t>Pct_long</t>
+  </si>
+  <si>
+    <t>Pct_short</t>
+  </si>
+  <si>
+    <t>Pct_medium</t>
+  </si>
+  <si>
+    <t>Rate
+Long</t>
+  </si>
+  <si>
+    <t>Rate
+Medium</t>
+  </si>
+  <si>
+    <t>Rate
+Short</t>
+  </si>
+  <si>
+    <t>Rate
+Group</t>
+  </si>
+  <si>
+    <t>Rent_group</t>
+  </si>
+  <si>
+    <t>Income</t>
+  </si>
+  <si>
+    <t>Mgmt Fee</t>
+  </si>
+  <si>
+    <t>Revpob</t>
+  </si>
+  <si>
+    <t>Revpab</t>
+  </si>
+  <si>
+    <t>MPR per bed</t>
+  </si>
+  <si>
+    <t>%
+Mgmt Fee</t>
+  </si>
+  <si>
+    <t>Reinvoices</t>
+  </si>
+  <si>
+    <t>Current
+Long</t>
+  </si>
+  <si>
+    <t>Current
+Medium</t>
+  </si>
+  <si>
+    <t>Current
+Short</t>
+  </si>
+  <si>
+    <t>Current
+Group</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0%;[Red]\-#,##0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -179,6 +239,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -206,7 +271,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -267,10 +332,37 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
         <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom/>
@@ -282,21 +374,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="15" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -308,6 +396,32 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="15" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="8" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -711,17 +825,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" style="2" customWidth="1"/>
-    <col min="2" max="3" width="14.140625" style="1" customWidth="1"/>
-    <col min="4" max="13" width="11.85546875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="10.28515625" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="14.42578125" style="1"/>
+    <col min="2" max="2" width="14.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" style="1" customWidth="1"/>
+    <col min="4" max="27" width="11.85546875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="14.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:28" s="11" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -729,105 +844,199 @@
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="M1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J1" s="3" t="s">
+      <c r="N1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="N1" s="12" t="e">
+      <c r="Q1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="R1" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="S1" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="U1" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="X1" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA1" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB1" s="8" t="e">
         <f>YEAR(A3)</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:28" ht="14.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="L2" s="26"/>
+      <c r="M2" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="O2" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="P2" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>10</v>
-      </c>
+      <c r="Q2" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" s="28"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="28"/>
+      <c r="V2" s="26"/>
+      <c r="W2" s="26"/>
+      <c r="X2" s="28"/>
+      <c r="Y2" s="26"/>
+      <c r="Z2" s="26"/>
+      <c r="AA2" s="30"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="14">
-        <f>1-SUM(E3:G3)</f>
+      <c r="B3" s="7"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="10">
+        <f>1-SUM(I3:K3)</f>
         <v>1</v>
       </c>
-      <c r="I3" s="8"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="11"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="20">
+        <f>C3*D3*SUMPRODUCT(E3:H3,I3:L3)*(1-M3)</f>
+        <v>0</v>
+      </c>
+      <c r="S3" s="23"/>
+      <c r="T3" s="22">
+        <f>IF(OR(LEFT(B3,6)="PFC002",LEFT(B3,6)="SAR326"),R3/1.1*S3,R3*S3)</f>
+        <v>0</v>
+      </c>
+      <c r="U3" s="21">
+        <f>IF(C3*D3,R3/(C3*D3),0)</f>
+        <v>0</v>
+      </c>
+      <c r="V3" s="15">
+        <f>IF(C3,R3/C3,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W3" s="24">
+        <f>SUMPRODUCT(E3:H3,I3:L3)</f>
+        <v>0</v>
+      </c>
+      <c r="X3" s="18"/>
+      <c r="Y3" s="19"/>
+      <c r="Z3" s="21"/>
+      <c r="AA3" s="24"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AA1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="A3:M99999">
+  <conditionalFormatting sqref="A3:AA99999">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$A2&gt;$A3</formula>
     </cfRule>
@@ -835,7 +1044,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <ignoredErrors>
-    <ignoredError sqref="N1" evalError="1"/>
+    <ignoredError sqref="AB1" evalError="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Forecast with av beds
</commit_message>
<xml_diff>
--- a/app/templates/report/forecast.xlsx
+++ b/app/templates/report/forecast.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51DEE2AD-6704-4BCE-8251-1D6B539DB7E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47165AC0-996B-47CB-BDEB-1ED40CAE5D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Forecast" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Forecast!$A$1:$AA$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Forecast!$A$1:$AB$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>Resource</t>
   </si>
@@ -181,17 +181,21 @@
   <si>
     <t>Current
 Group</t>
+  </si>
+  <si>
+    <t>Available beds</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0%;[Red]\-#,##0%"/>
     <numFmt numFmtId="167" formatCode="#,##0.0\ &quot;€&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -374,7 +378,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -422,6 +426,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -825,18 +830,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="8.7109375" style="1" customWidth="1"/>
-    <col min="4" max="27" width="11.85546875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="14.42578125" style="1"/>
+    <col min="4" max="28" width="11.85546875" style="1" customWidth="1"/>
+    <col min="29" max="29" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="14.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="11" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" s="11" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -889,41 +894,44 @@
         <v>38</v>
       </c>
       <c r="R1" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="S1" s="14" t="s">
+      <c r="T1" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="14" t="s">
+      <c r="V1" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="14" t="s">
+      <c r="Y1" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="AA1" s="25" t="s">
+      <c r="AB1" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="AB1" s="8" t="e">
+      <c r="AC1" s="8" t="e">
         <f>YEAR(A3)</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="14.25" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A2" s="26" t="s">
         <v>10</v>
       </c>
@@ -974,17 +982,18 @@
         <v>38</v>
       </c>
       <c r="R2" s="28"/>
-      <c r="S2" s="26"/>
+      <c r="S2" s="28"/>
       <c r="T2" s="26"/>
-      <c r="U2" s="28"/>
-      <c r="V2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="28"/>
       <c r="W2" s="26"/>
-      <c r="X2" s="28"/>
-      <c r="Y2" s="26"/>
+      <c r="X2" s="26"/>
+      <c r="Y2" s="28"/>
       <c r="Z2" s="26"/>
-      <c r="AA2" s="30"/>
+      <c r="AA2" s="26"/>
+      <c r="AB2" s="30"/>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
@@ -1007,44 +1016,45 @@
       <c r="O3" s="31"/>
       <c r="P3" s="31"/>
       <c r="Q3" s="31"/>
-      <c r="R3" s="20">
+      <c r="R3" s="33"/>
+      <c r="S3" s="20">
         <f>C3*D3*SUMPRODUCT(E3:H3,I3:L3)*(1-M3)</f>
         <v>0</v>
       </c>
-      <c r="S3" s="23"/>
-      <c r="T3" s="22">
-        <f>IF(OR(LEFT(B3,6)="PFC002",LEFT(B3,6)="SAR326"),R3/1.1*S3,R3*S3)</f>
+      <c r="T3" s="23"/>
+      <c r="U3" s="22">
+        <f>IF(OR(LEFT(B3,6)="PFC002",LEFT(B3,6)="SAR326"),S3/1.1*T3,S3*T3)</f>
         <v>0</v>
       </c>
-      <c r="U3" s="21">
-        <f>IF(C3*D3,R3/(C3*D3),0)</f>
+      <c r="V3" s="21">
+        <f>IF(C3*D3,S3/(C3*D3),0)</f>
         <v>0</v>
       </c>
-      <c r="V3" s="15">
-        <f>IF(C3,R3/C3,0)</f>
+      <c r="W3" s="15">
+        <f>IF(C3,S3/C3,0)</f>
         <v>0</v>
       </c>
-      <c r="W3" s="24">
+      <c r="X3" s="24">
         <f>SUMPRODUCT(E3:H3,I3:L3)</f>
         <v>0</v>
       </c>
-      <c r="X3" s="18"/>
-      <c r="Y3" s="19"/>
-      <c r="Z3" s="21"/>
-      <c r="AA3" s="24"/>
+      <c r="Y3" s="18"/>
+      <c r="Z3" s="19"/>
+      <c r="AA3" s="21"/>
+      <c r="AB3" s="24"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AB1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="A3:AA99999">
+  <conditionalFormatting sqref="A3:AB99999">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$A2&gt;$A3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="AB1" evalError="1"/>
+    <ignoredError sqref="AC1" evalError="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>